<commit_message>
Variant 3: swap the open Graph slot for videographer Асанов; retitle Жанабеков
In variant 3, replace the empty Graph position with Асанов Әділ Асанұлы
(Видеограф/видеомонтажер, 1 000 162 ₸) and rename Жанабеков's box from
«Мобилограф / монтажёр Sport» to «Видеограф Sport». Продакшн is now
11 086 553 ₸; grand total 39 218 833 ₸ (34 people). Adds an OVERRIDE_FILE
env to make_xlsx.py for per-field overrides (build/v3_overrides.json).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015FvdqNtbbJPjugTChUgZkw
</commit_message>
<xml_diff>
--- a/Данные — вариант 3.xlsx
+++ b/Данные — вариант 3.xlsx
@@ -1752,18 +1752,18 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Graph</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr"/>
-      <c r="G29" s="10" t="n">
-        <v>940000</v>
-      </c>
-      <c r="H29" s="9" t="inlineStr">
-        <is>
-          <t>макс.</t>
-        </is>
-      </c>
+          <t>Видеограф/видеомонтажер</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Асанов Әділ Асанұлы</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>1000162</v>
+      </c>
+      <c r="H29" s="9" t="inlineStr"/>
       <c r="I29" s="9" t="inlineStr"/>
       <c r="J29" s="5" t="inlineStr">
         <is>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Мобилограф / монтажёр Sport</t>
+          <t>Видеограф Sport</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">

</xml_diff>